<commit_message>
Se registró el cierre en producción y la base de datos con sus evidencias
</commit_message>
<xml_diff>
--- a/docs/assets/infraestructura/s1-e2-matriz-componentes-dimensionamiento.xlsx
+++ b/docs/assets/infraestructura/s1-e2-matriz-componentes-dimensionamiento.xlsx
@@ -516,7 +516,7 @@
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
     <col min="5" max="5" width="59.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="59.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1252,7 +1252,7 @@
         <v>Crítica</v>
       </c>
       <c r="G32" t="str">
-        <v>Implementado (reglas corregidas sin publicar)</v>
+        <v>Implementado (reglas corregidas publicadas el 2026-10-24)</v>
       </c>
     </row>
     <row r="33">

</xml_diff>